<commit_message>
CB fix: PO data mapping update
</commit_message>
<xml_diff>
--- a/data/input/In_Transit_PO data.xlsx
+++ b/data/input/In_Transit_PO data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Nitesh\AM - Inventory replenishment\AM_Replenishment\data\input\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{92067E61-E66A-49E6-98EB-3B8D74A2B273}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2E52AD55-9B90-4DE6-82FB-A612D2B27D24}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{ED1C42A4-610F-4493-A647-7EDE7899E1B2}"/>
   </bookViews>
@@ -16,12 +16,21 @@
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$P$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$P$63</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
@@ -3900,7 +3909,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:P1" xr:uid="{AD5A3FE4-F9D3-480E-B305-3F537BEA10CA}"/>
+  <autoFilter ref="A1:P63" xr:uid="{AD5A3FE4-F9D3-480E-B305-3F537BEA10CA}"/>
   <conditionalFormatting sqref="B2:B63">
     <cfRule type="duplicateValues" dxfId="0" priority="2"/>
   </conditionalFormatting>

</xml_diff>